<commit_message>
Add American Diploma equivalent percentage calculation
Adds an equivalent percentage field derived from SAT I/II and GPA
per the government universities coordination office formula, plus
supporting migration and export/UI updates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/StudentRegistry.API/Templates/StudentExportTemplate.xlsx
+++ b/backend/StudentRegistry.API/Templates/StudentExportTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohmm\Documents\GitHub\dynamic--form-based-web-application\backend\StudentRegistry.API\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDF564F-590D-444C-9DA2-3CC314E69613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0A7CC1-6DB1-4305-8920-2EC08A3419EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>بيانات ولي أمر الطالب</t>
   </si>
@@ -31,18 +31,6 @@
     <t>اسم الطالب من واقع شهادة الميلاد :</t>
   </si>
   <si>
-    <t>الرقم القومي :</t>
-  </si>
-  <si>
-    <t>رقم التليفون أرضي :</t>
-  </si>
-  <si>
-    <t>عنوان الطالب :</t>
-  </si>
-  <si>
-    <t>مركز :</t>
-  </si>
-  <si>
     <t>النوع (ذكر / أنثى) :</t>
   </si>
   <si>
@@ -52,37 +40,10 @@
     <t>مجموع الطالب في الثانوية العامة :</t>
   </si>
   <si>
-    <t>الشعبة :</t>
-  </si>
-  <si>
     <t>المدرسة الحاصل منها على الثانوية العامة :</t>
   </si>
   <si>
     <t>سنة الحصول على الثانوية العامة أو ما يعادلها :</t>
-  </si>
-  <si>
-    <t>محافظة الميلاد :</t>
-  </si>
-  <si>
-    <t>محل الميلاد :</t>
-  </si>
-  <si>
-    <t>محافظة :</t>
-  </si>
-  <si>
-    <t>رقم الموبايل :</t>
-  </si>
-  <si>
-    <t>رقم التليفون :</t>
-  </si>
-  <si>
-    <t>العنوان بالتفصيل :</t>
-  </si>
-  <si>
-    <t>اسم ولي الأمر :</t>
-  </si>
-  <si>
-    <t>وظيفته :</t>
   </si>
   <si>
     <t xml:space="preserve">                                  وثيقة تعارف (2026/2027م)</t>
@@ -109,6 +70,39 @@
       </rPr>
       <t>بيانات الطالب</t>
     </r>
+  </si>
+  <si>
+    <t>رقم الهاتف :</t>
+  </si>
+  <si>
+    <t>الـــــرقم القـــــومـــــي :</t>
+  </si>
+  <si>
+    <t>رقم التليفون أرضـــــي :</t>
+  </si>
+  <si>
+    <t>عـــــنـــــوان الطالـــــب :</t>
+  </si>
+  <si>
+    <t>محـــــل المـــــيلاد :</t>
+  </si>
+  <si>
+    <t>الشـــــعـــــبة :</t>
+  </si>
+  <si>
+    <t>اســـــم ولي الأمـــــر :</t>
+  </si>
+  <si>
+    <t>وظــــــــــيفته :</t>
+  </si>
+  <si>
+    <t>الرقـــــم القومـــــي :</t>
+  </si>
+  <si>
+    <t>الـــــعنوان بالتفصيل :</t>
+  </si>
+  <si>
+    <t>رقـــــم الهاتف :</t>
   </si>
 </sst>
 </file>
@@ -221,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -248,6 +242,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -261,15 +261,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1378,11 +1369,11 @@
     </row>
     <row r="2" spans="1:5" ht="67.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
-      <c r="B2" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
+      <c r="B2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
       <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:5" ht="46.8" customHeight="1" x14ac:dyDescent="0.35">
@@ -1395,7 +1386,7 @@
     <row r="4" spans="1:5" ht="73.8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="7" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -1406,107 +1397,100 @@
       <c r="B5" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
+        <v>10</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="6" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E7" s="6"/>
     </row>
     <row r="8" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
+        <v>12</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="16"/>
+        <v>13</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="6" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C10" s="6"/>
-      <c r="D10" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="E10" s="6"/>
     </row>
     <row r="11" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C11" s="6"/>
-      <c r="D11" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="D11" s="6"/>
       <c r="E11" s="6"/>
     </row>
     <row r="12" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
+        <v>4</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
     </row>
     <row r="13" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
+        <v>14</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
     </row>
     <row r="14" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="16" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
@@ -1517,58 +1501,56 @@
     </row>
     <row r="17" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
     </row>
     <row r="18" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
+        <v>16</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
     </row>
     <row r="20" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
+        <v>17</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
     </row>
     <row r="21" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
+        <v>18</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C22" s="6"/>
-      <c r="D22" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="D22" s="6"/>
       <c r="E22" s="6"/>
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1608,11 +1590,7 @@
       <c r="E27"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="C8:E8"/>
+  <mergeCells count="17">
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="C12:E12"/>
@@ -1622,8 +1600,13 @@
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="C8:E8"/>
     <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C18:E18"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>